<commit_message>
Formula to find Dormants
</commit_message>
<xml_diff>
--- a/JobHunt/sample-jobhunt.xlsx
+++ b/JobHunt/sample-jobhunt.xlsx
@@ -1,15 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\arun\Learn\Excels\JobHunt\JobHunt\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE39539-920C-4C29-8938-6AFB484AC63F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="JobHunt" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -30,12 +52,113 @@
 </metadata>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+  <si>
+    <t>Company Name</t>
+  </si>
+  <si>
+    <t>Position Name</t>
+  </si>
+  <si>
+    <t>Role Type</t>
+  </si>
+  <si>
+    <t>Date- Job Posted</t>
+  </si>
+  <si>
+    <t>Date- Applied</t>
+  </si>
+  <si>
+    <t>Flag to see if the job posting is still accepting candidates</t>
+  </si>
+  <si>
+    <t>Date- Short Listed</t>
+  </si>
+  <si>
+    <t>Date- Interview/Test</t>
+  </si>
+  <si>
+    <t>Date- Offer</t>
+  </si>
+  <si>
+    <t>Date- Rejected</t>
+  </si>
+  <si>
+    <t>Date- Declined by Me</t>
+  </si>
+  <si>
+    <t>Log</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Portal</t>
+  </si>
+  <si>
+    <t>Acme Corp</t>
+  </si>
+  <si>
+    <t>Project Manager</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/1/</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Phone screen scheduled.</t>
+  </si>
+  <si>
+    <t>Beta Ltd</t>
+  </si>
+  <si>
+    <t>Program Manager</t>
+  </si>
+  <si>
+    <t>https://jobs.example.com/a</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>20260510: Rejected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URL of Job Posting </t>
+  </si>
+  <si>
+    <t>AI Engineer</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/2/</t>
+  </si>
+  <si>
+    <t>https://jobs.example.com/b</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/jobs/view/3/</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>Center Head</t>
+  </si>
+  <si>
+    <t>Head</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -43,16 +166,49 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,19 +216,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -397,132 +584,280 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.75" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Company Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Position Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Role Type</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Date- Job Posted</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Date- Applied</v>
-      </c>
-      <c r="F1" t="str">
-        <v>URL of Job Posting</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Flag to see if the job posting is still accepting candidates</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Date- Short Listed</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Date- Interview/Test</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Date- Offer</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Date- Rejected</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Date- Declined by Me</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Log</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="O1" t="str">
-        <v>Portal</v>
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Acme Corp</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Project Manager</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Delivery</v>
-      </c>
-      <c r="D2" s="1">
+    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="7">
         <v>46143.333333333336</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="7">
         <v>46145.333333333336</v>
       </c>
-      <c r="F2" t="str">
-        <v>https://www.linkedin.com/jobs/view/1/</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="H2" s="1">
+      <c r="F2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="7">
         <v>46147.333333333336</v>
       </c>
-      <c r="M2" t="str">
-        <v>Phone screen scheduled.</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Short listed</v>
-      </c>
-      <c r="O2" t="str">
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N2" s="5" t="str" cm="1">
+        <f t="array" aca="1" ref="N2" ca="1">_xlfn.LET(_xlpm.stateName,SUBSTITUTE(_xlfn.IFS(ISNUMBER(L2),$L$1,ISNUMBER(K2),$K$1, ISNUMBER(J2),$J$1,ISNUMBER(I2),$I$1, ISNUMBER(H2),$H$1, ISNUMBER(E2),$E$1),"Date- ",""),
+     _xlpm.age,_xlfn.DAYS(TODAY(),_xlfn.IFS(ISNUMBER(I2),I2,ISNUMBER(H2),H2,ISNUMBER(E2),E2)),
+     IF(AND(_xlpm.age&gt;30, _xlpm.stateName="Applied"),"Dormant",_xlpm.stateName))</f>
+        <v>Short Listed</v>
+      </c>
+      <c r="O2" s="6" t="str">
+        <f>SUBSTITUTE(SUBSTITUTE(MID(F2, FIND("://", F2) + 3, IF(ISNUMBER(FIND("/", F2, 9)), FIND("/", F2, 9), LEN(F2)+1) - FIND("://", F2) - 3), "www.", ""), ".com", "")</f>
         <v>linkedin</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Beta Ltd</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Program Manager</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Delivery</v>
-      </c>
-      <c r="D3" s="1">
+    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="7">
         <v>46144.333333333336</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="7">
         <v>46146.333333333336</v>
       </c>
-      <c r="F3" t="str">
-        <v>https://jobs.example.com/a</v>
-      </c>
-      <c r="G3" t="str">
-        <v>No</v>
-      </c>
-      <c r="I3" s="1">
+      <c r="F3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3" s="7">
         <v>46150.333333333336</v>
       </c>
-      <c r="K3" s="1">
+      <c r="J3" s="5"/>
+      <c r="K3" s="7">
         <v>46152.333333333336</v>
       </c>
-      <c r="M3" t="str">
-        <v>20260510: Rejected</v>
-      </c>
-      <c r="N3" t="str">
+      <c r="L3" s="5"/>
+      <c r="M3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="5" t="str" cm="1">
+        <f t="array" aca="1" ref="N3" ca="1">_xlfn.LET(_xlpm.stateName,SUBSTITUTE(_xlfn.IFS(ISNUMBER(L3),$L$1,ISNUMBER(K3),$K$1, ISNUMBER(J3),$J$1,ISNUMBER(I3),$I$1, ISNUMBER(H3),$H$1, ISNUMBER(E3),$E$1),"Date- ",""),
+     _xlpm.age,_xlfn.DAYS(TODAY(),_xlfn.IFS(ISNUMBER(I3),I3,ISNUMBER(H3),H3,ISNUMBER(E3),E3)),
+     IF(AND(_xlpm.age&gt;30, _xlpm.stateName="Applied"),"Dormant",_xlpm.stateName))</f>
         <v>Rejected</v>
       </c>
-      <c r="O3" t="str">
-        <v>example</v>
+      <c r="O3" s="6" t="str">
+        <f>SUBSTITUTE(SUBSTITUTE(MID(F3, FIND("://", F3) + 3, IF(ISNUMBER(FIND("/", F3, 9)), FIND("/", F3, 9), LEN(F3)+1) - FIND("://", F3) - 3), "www.", ""), ".com", "")</f>
+        <v>jobs.example</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="7">
+        <v>46145</v>
+      </c>
+      <c r="E4" s="7">
+        <v>46147</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N4" s="5" t="str" cm="1">
+        <f t="array" aca="1" ref="N4" ca="1">_xlfn.LET(_xlpm.stateName,SUBSTITUTE(_xlfn.IFS(ISNUMBER(L4),$L$1,ISNUMBER(K4),$K$1, ISNUMBER(J4),$J$1,ISNUMBER(I4),$I$1, ISNUMBER(H4),$H$1, ISNUMBER(E4),$E$1),"Date- ",""),
+     _xlpm.age,_xlfn.DAYS(TODAY(),_xlfn.IFS(ISNUMBER(I4),I4,ISNUMBER(H4),H4,ISNUMBER(E4),E4)),
+     IF(AND(_xlpm.age&gt;30, _xlpm.stateName="Applied"),"Dormant",_xlpm.stateName))</f>
+        <v>Applied</v>
+      </c>
+      <c r="O4" s="6" t="str">
+        <f t="shared" ref="O4:O6" si="0">SUBSTITUTE(SUBSTITUTE(MID(F4, FIND("://", F4) + 3, IF(ISNUMBER(FIND("/", F4, 9)), FIND("/", F4, 9), LEN(F4)+1) - FIND("://", F4) - 3), "www.", ""), ".com", "")</f>
+        <v>linkedin</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="7">
+        <v>46142</v>
+      </c>
+      <c r="E5" s="7">
+        <v>46151</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="5" t="str" cm="1">
+        <f t="array" aca="1" ref="N5" ca="1">_xlfn.LET(_xlpm.stateName,SUBSTITUTE(_xlfn.IFS(ISNUMBER(L5),$L$1,ISNUMBER(K5),$K$1, ISNUMBER(J5),$J$1,ISNUMBER(I5),$I$1, ISNUMBER(H5),$H$1, ISNUMBER(E5),$E$1),"Date- ",""),
+     _xlpm.age,_xlfn.DAYS(TODAY(),_xlfn.IFS(ISNUMBER(I5),I5,ISNUMBER(H5),H5,ISNUMBER(E5),E5)),
+     IF(AND(_xlpm.age&gt;30, _xlpm.stateName="Applied"),"Dormant",_xlpm.stateName))</f>
+        <v>Applied</v>
+      </c>
+      <c r="O5" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>jobs.example</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="7">
+        <v>46142</v>
+      </c>
+      <c r="E6" s="7">
+        <v>46143</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="7"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="N6" s="5" t="str" cm="1">
+        <f t="array" aca="1" ref="N6" ca="1">_xlfn.LET(_xlpm.stateName,SUBSTITUTE(_xlfn.IFS(ISNUMBER(L6),$L$1,ISNUMBER(K6),$K$1, ISNUMBER(J6),$J$1,ISNUMBER(I6),$I$1, ISNUMBER(H6),$H$1, ISNUMBER(E6),$E$1),"Date- ",""),
+     _xlpm.age,_xlfn.DAYS(TODAY(),_xlfn.IFS(ISNUMBER(I6),I6,ISNUMBER(H6),H6,ISNUMBER(E6),E6)),
+     IF(AND(_xlpm.age&gt;30, _xlpm.stateName="Applied"),"Dormant",_xlpm.stateName))</f>
+        <v>Dormant</v>
+      </c>
+      <c r="O6" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>linkedin</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
+    <ignoredError sqref="A3:B3 A2:B2 G3:M3 G2:M2 D2:E2 D3:E3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>